<commit_message>
Rebalance Career Courage scoring and add challenge copy variety
Career Courage had 3 of 6 questions scored as binary Yes/No, giving it
roughly double the score variance of every other category and structurally
favoring it to be flagged as the weakest/challenge category (~19% vs an
~11% fair share across 20k simulated runs). Converted KA001/KA004/KA007 to
5-point frequency scales to match the rest of the bank, in both
data/questions.js and the Excel source of truth.

Also expanded challengeBank and achievementChallenges from one fixed line
per tier to 3 randomized variants each, so retaking the quiz doesn't
surface the exact same challenge text every time.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ballsy_Questions_V4_English.xlsx
+++ b/Ballsy_Questions_V4_English.xlsx
@@ -57,7 +57,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +80,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -163,6 +169,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -253,6 +260,41 @@
     <comment ref="E6" authorId="0" shapeId="0">
       <text>
         <t>Corrected 5-1 -&gt; 1-5. Hesitating 'often' without acting is the fearful answer; it was scoring highest instead of lowest.</t>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0" shapeId="0">
+      <text>
+        <t>Rebalanced from binary Yes/No to 5-point scale (2026-08-14): Career Courage had 3 of 6 questions as binary, giving it ~2x the variance of other categories and structurally favoring it to appear as the weakest/challenge category. Converted to match the 5-point-scale convention used elsewhere in the bank.</t>
+      </text>
+    </comment>
+    <comment ref="E22" authorId="0" shapeId="0">
+      <text>
+        <t>Rebalanced from binary Yes/No to 5-point scale (2026-08-14): Career Courage had 3 of 6 questions as binary, giving it ~2x the variance of other categories and structurally favoring it to appear as the weakest/challenge category. Converted to match the 5-point-scale convention used elsewhere in the bank.</t>
+      </text>
+    </comment>
+    <comment ref="D23" authorId="0" shapeId="0">
+      <text>
+        <t>Rebalanced from binary Yes/No to 5-point scale (2026-08-14): Career Courage had 3 of 6 questions as binary, giving it ~2x the variance of other categories and structurally favoring it to appear as the weakest/challenge category. Converted to match the 5-point-scale convention used elsewhere in the bank.</t>
+      </text>
+    </comment>
+    <comment ref="E23" authorId="0" shapeId="0">
+      <text>
+        <t>Rebalanced from binary Yes/No to 5-point scale (2026-08-14): Career Courage had 3 of 6 questions as binary, giving it ~2x the variance of other categories and structurally favoring it to appear as the weakest/challenge category. Converted to match the 5-point-scale convention used elsewhere in the bank.</t>
+      </text>
+    </comment>
+    <comment ref="C25" authorId="0" shapeId="0">
+      <text>
+        <t>Rebalanced from binary Yes/No to 5-point scale (2026-08-14): Career Courage had 3 of 6 questions as binary, giving it ~2x the variance of other categories and structurally favoring it to appear as the weakest/challenge category. Converted to match the 5-point-scale convention used elsewhere in the bank.</t>
+      </text>
+    </comment>
+    <comment ref="D25" authorId="0" shapeId="0">
+      <text>
+        <t>Rebalanced from binary Yes/No to 5-point scale (2026-08-14): Career Courage had 3 of 6 questions as binary, giving it ~2x the variance of other categories and structurally favoring it to appear as the weakest/challenge category. Converted to match the 5-point-scale convention used elsewhere in the bank.</t>
+      </text>
+    </comment>
+    <comment ref="E25" authorId="0" shapeId="0">
+      <text>
+        <t>Rebalanced from binary Yes/No to 5-point scale (2026-08-14): Career Courage had 3 of 6 questions as binary, giving it ~2x the variance of other categories and structurally favoring it to appear as the weakest/challenge category. Converted to match the 5-point-scale convention used elsewhere in the bank.</t>
       </text>
     </comment>
     <comment ref="E37" authorId="0" shapeId="0">
@@ -1370,14 +1412,14 @@
           <t>I apply for positions even when I do not meet all the requirements.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Yes/No</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>1-5</t>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Very often, Often, Neutral, Rarely, Very rarely</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>5-1</t>
         </is>
       </c>
       <c r="F22" s="11" t="n">
@@ -1403,14 +1445,14 @@
           <t>I can hold a strong opinion on an issue even when I am unsure whether I am right.</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Yes/No</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>1-5</t>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Very often, Often, Neutral, Rarely, Very rarely</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>5-1</t>
         </is>
       </c>
       <c r="F23" s="11" t="n">
@@ -1464,14 +1506,19 @@
           <t>Career Courage</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Have you ever stayed in a job primarily because it felt safe?</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Yes/No</t>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>I stay in jobs primarily because they feel safe.</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Very often, Often, Neutral, Rarely, Very rarely</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>1-5</t>
         </is>
       </c>
       <c r="F25" s="11" t="n">
@@ -4007,6 +4054,7 @@
         <v/>
       </c>
     </row>
+    <row r="110"/>
     <row r="111" ht="30.05" customHeight="1">
       <c r="C111" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rework L006 and remove L007 from Life Courage
L006's phrasing was broken ("Dare you to start over?") and L007
overlapped heavily with L001/L005's change-related questions, per user
feedback. Reworded L006 to a distinct angle (walking away from something
stable) and dropped L007 entirely, in both data/questions.js and the
Excel source of truth.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ballsy_Questions_V4_English.xlsx
+++ b/Ballsy_Questions_V4_English.xlsx
@@ -392,12 +392,17 @@
         <t>Corrected text. Original text had no referent ('this' pointed to nothing) and was ambiguous out of context; reworded to stand on its own while keeping the same scoring direction (5-1) and options.</t>
       </text>
     </comment>
-    <comment ref="E98" authorId="0" shapeId="0">
+    <comment ref="C95" authorId="0" shapeId="0">
+      <text>
+        <t>Reworded (2026-08-17): replaced awkward/vague phrasing per user feedback, and to reduce overlap with L001/L005.</t>
+      </text>
+    </comment>
+    <comment ref="E97" authorId="0" shapeId="0">
       <text>
         <t>Corrected Analysis -&gt; 5-1. Source sheet left this undecided ('Analysis'); the app guessed asc (1-5). 'Something that's holding me back' is the worst answer and should score lowest, so it should be desc (5-1).</t>
       </text>
     </comment>
-    <comment ref="E107" authorId="0" shapeId="0">
+    <comment ref="E106" authorId="0" shapeId="0">
       <text>
         <t>Corrected 5-1 -&gt; 1-5. 'Almost everything' controlled by others' expectations is the least autonomous/brave answer; it was scoring highest instead of lowest.</t>
       </text>
@@ -727,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.05"/>
   <cols>
     <col width="15.33203125" customWidth="1" min="2" max="2"/>
@@ -3641,9 +3646,9 @@
           <t>Life Courage</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Dare you to start over?</t>
+      <c r="C95" s="17" t="inlineStr">
+        <is>
+          <t>Would you walk away from something stable if you knew, deep down, it wasn't right for you?</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
@@ -3666,7 +3671,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>L007</t>
+          <t>L008</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3676,30 +3681,30 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>You get the opportunity to start completely over. New city. New job. New people. What do you feel first?</t>
+          <t>Which conversation do you know you should have?</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Frykt, Motstand, Usikker nysgjerrighet, Spenning, Begeistring</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>1-5</t>
+          <t>Fritekst + AI-kategorisering</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="F96" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G96" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>L008</t>
+          <t>L009</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3709,71 +3714,71 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Which conversation do you know you should have?</t>
+          <t>What would the people closest to you say you are afraid of?</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>Fritekst + AI-kategorisering</t>
-        </is>
-      </c>
-      <c r="E97" s="7" t="inlineStr">
-        <is>
-          <t>Analysis</t>
+          <t>Vet ikke, En liten ting, Flere mindre ting, Én stor ting, Noe som holder meg tilbake</t>
+        </is>
+      </c>
+      <c r="E97" s="16" t="inlineStr">
+        <is>
+          <t>5-1</t>
         </is>
       </c>
       <c r="F97" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G97" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="98" ht="30.05" customHeight="1">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>L009</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Life Courage</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>What would the people closest to you say you are afraid of?</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>Vet ikke, En liten ting, Flere mindre ting, Én stor ting, Noe som holder meg tilbake</t>
-        </is>
-      </c>
-      <c r="E98" s="16" t="inlineStr">
-        <is>
-          <t>5-1</t>
-        </is>
-      </c>
-      <c r="F98" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G98" s="6" t="n">
-        <v>5</v>
+      <c r="F98" s="10" t="n"/>
+      <c r="H98" s="13" t="inlineStr">
+        <is>
+          <t>Category Subtotal</t>
+        </is>
       </c>
     </row>
     <row r="99">
-      <c r="F99" s="10" t="n"/>
-      <c r="H99" s="13" t="inlineStr">
-        <is>
-          <t>Category Subtotal</t>
-        </is>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>FP001</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Fear Profile</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>What do you fear most?</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>Rejection, Criticism, Loneliness, Failure, Loss of control</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>All options give 3 points</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G99" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>FP001</t>
+          <t>FP002</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3783,17 +3788,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>What do you fear most?</t>
+          <t>Rejection</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>Rejection, Criticism, Loneliness, Failure, Loss of control</t>
-        </is>
-      </c>
-      <c r="E100" s="7" t="inlineStr">
-        <is>
-          <t>All options give 3 points</t>
+          <t>Strongly agree, Somewhat agree, Neutral, Somewhat disagree, Strongly disagree</t>
+        </is>
+      </c>
+      <c r="E100" s="9" t="inlineStr">
+        <is>
+          <t>5-1</t>
         </is>
       </c>
       <c r="F100" s="5" t="n">
@@ -3806,7 +3811,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FP002</t>
+          <t>FP003</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3816,7 +3821,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Rejection</t>
+          <t>Criticism</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -3839,7 +3844,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>FP003</t>
+          <t>FP004</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3849,7 +3854,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Criticism</t>
+          <t>Loneliness</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -3863,16 +3868,16 @@
         </is>
       </c>
       <c r="F102" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G102" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>FP004</t>
+          <t>FP005</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3882,7 +3887,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Loneliness</t>
+          <t>Failure</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -3896,16 +3901,16 @@
         </is>
       </c>
       <c r="F103" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G103" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>FP005</t>
+          <t>FP006</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3915,17 +3920,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Failure</t>
+          <t>I do not need other people's approval to act.</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>Strongly agree, Somewhat agree, Neutral, Somewhat disagree, Strongly disagree</t>
-        </is>
-      </c>
-      <c r="E104" s="9" t="inlineStr">
-        <is>
-          <t>5-1</t>
+          <t>Strongly disagree, Somewhat disagree, Neutral, Somewhat agree, Strongly agree</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>1-5</t>
         </is>
       </c>
       <c r="F104" s="5" t="n">
@@ -3938,7 +3943,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>FP006</t>
+          <t>FP007</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3948,7 +3953,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>I do not need other people's approval to act.</t>
+          <t>I am comfortable with not being liked by everyone.</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
@@ -3971,7 +3976,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>FP007</t>
+          <t>FP008</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3981,15 +3986,15 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>I am comfortable with not being liked by everyone.</t>
+          <t>How much of your life is controlled by other people's expectations?</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>Strongly disagree, Somewhat disagree, Neutral, Somewhat agree, Strongly agree</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
+          <t>Nesten alt, Mye, Noe, Lite, Nesten ingenting</t>
+        </is>
+      </c>
+      <c r="E106" s="15" t="inlineStr">
         <is>
           <t>1-5</t>
         </is>
@@ -4002,78 +4007,45 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>FP008</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Fear Profile</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>How much of your life is controlled by other people's expectations?</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>Nesten alt, Mye, Noe, Lite, Nesten ingenting</t>
-        </is>
-      </c>
-      <c r="E107" s="15" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
-      <c r="F107" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="G107" s="5" t="n">
-        <v>5</v>
+      <c r="F107" s="10" t="n"/>
+      <c r="H107" s="13" t="inlineStr">
+        <is>
+          <t>Category Subtotal</t>
+        </is>
       </c>
     </row>
     <row r="108">
-      <c r="F108" s="10" t="n"/>
-      <c r="H108" s="13" t="inlineStr">
-        <is>
-          <t>Category Subtotal</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="B109" t="n">
+      <c r="B108" t="n">
         <v>11</v>
       </c>
-      <c r="C109" t="n">
+      <c r="C108" t="n">
         <v>3</v>
       </c>
-      <c r="D109">
+      <c r="D108">
         <f>B109*C109</f>
         <v/>
       </c>
     </row>
-    <row r="110"/>
+    <row r="109"/>
+    <row r="110">
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Ballsy Score-formel</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Question score (1-5) × Question Weight × Difficulty = Ballsy Subscore</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Total Score</t>
+        </is>
+      </c>
+    </row>
     <row r="111" ht="30.05" customHeight="1">
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Ballsy Score-formel</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>Question score (1-5) × Question Weight × Difficulty = Ballsy Subscore</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>Total Score</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="D112" t="inlineStr">
+      <c r="D111" t="inlineStr">
         <is>
           <t>Average of Top 3 Categories = Ballsy Types</t>
         </is>

</xml_diff>